<commit_message>
test: improve date, financial, info conformance fixtures with edge cases
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/date/date_math.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/date/date_math.xlsx
@@ -20,18 +20,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t xml:space="preserve">date_serial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">edate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eomonth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">datedif</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t xml:space="preserve">serial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">edate_3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">edate_neg2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eomonth_0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eomonth_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">datedif_days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">datedif_months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">datedif_years</t>
   </si>
 </sst>
 </file>
@@ -304,7 +316,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -320,6 +332,18 @@
       <c r="D1" s="0" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="n">
@@ -330,12 +354,28 @@
         <v>45092</v>
       </c>
       <c r="C2" s="0" t="n">
+        <f aca="false">EDATE(A2,-2)</f>
+        <v>44941</v>
+      </c>
+      <c r="D2" s="0" t="n">
         <f aca="false">EOMONTH(A2,0)</f>
         <v>45016</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="E2" s="0" t="n">
+        <f aca="false">EOMONTH(A2,1)</f>
+        <v>45046</v>
+      </c>
+      <c r="F2" s="0" t="n">
         <f aca="false">DATEDIF(DATE(2020,1,1),A2,"d")</f>
         <v>1169</v>
+      </c>
+      <c r="G2" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A2,"m")</f>
+        <v>38</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A2,"y")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -347,29 +387,61 @@
         <v>45122</v>
       </c>
       <c r="C3" s="0" t="n">
+        <f aca="false">EDATE(A3,-2)</f>
+        <v>44972</v>
+      </c>
+      <c r="D3" s="0" t="n">
         <f aca="false">EOMONTH(A3,0)</f>
         <v>45046</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="E3" s="0" t="n">
+        <f aca="false">EOMONTH(A3,1)</f>
+        <v>45077</v>
+      </c>
+      <c r="F3" s="0" t="n">
         <f aca="false">DATEDIF(DATE(2020,1,1),A3,"d")</f>
         <v>1200</v>
       </c>
+      <c r="G3" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A3,"m")</f>
+        <v>39</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A3,"y")</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="n">
-        <v>45061</v>
+        <v>45100</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">EDATE(A4,3)</f>
-        <v>45153</v>
+        <v>45192</v>
       </c>
       <c r="C4" s="0" t="n">
+        <f aca="false">EDATE(A4,-2)</f>
+        <v>45039</v>
+      </c>
+      <c r="D4" s="0" t="n">
         <f aca="false">EOMONTH(A4,0)</f>
-        <v>45077</v>
-      </c>
-      <c r="D4" s="0" t="n">
+        <v>45107</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <f aca="false">EOMONTH(A4,1)</f>
+        <v>45138</v>
+      </c>
+      <c r="F4" s="0" t="n">
         <f aca="false">DATEDIF(DATE(2020,1,1),A4,"d")</f>
-        <v>1230</v>
+        <v>1269</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A4,"m")</f>
+        <v>41</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A4,"y")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -381,12 +453,28 @@
         <v>45017</v>
       </c>
       <c r="C5" s="0" t="n">
+        <f aca="false">EDATE(A5,-2)</f>
+        <v>44866</v>
+      </c>
+      <c r="D5" s="0" t="n">
         <f aca="false">EOMONTH(A5,0)</f>
         <v>44957</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="E5" s="0" t="n">
+        <f aca="false">EOMONTH(A5,1)</f>
+        <v>44985</v>
+      </c>
+      <c r="F5" s="0" t="n">
         <f aca="false">DATEDIF(DATE(2020,1,1),A5,"d")</f>
         <v>1096</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A5,"m")</f>
+        <v>36</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A5,"y")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -398,97 +486,127 @@
         <v>45292</v>
       </c>
       <c r="C6" s="0" t="n">
+        <f aca="false">EDATE(A6,-2)</f>
+        <v>45139</v>
+      </c>
+      <c r="D6" s="0" t="n">
         <f aca="false">EOMONTH(A6,0)</f>
         <v>45230</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="E6" s="0" t="n">
+        <f aca="false">EOMONTH(A6,1)</f>
+        <v>45260</v>
+      </c>
+      <c r="F6" s="0" t="n">
         <f aca="false">DATEDIF(DATE(2020,1,1),A6,"d")</f>
         <v>1369</v>
       </c>
+      <c r="G6" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A6,"m")</f>
+        <v>45</v>
+      </c>
+      <c r="H6" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A6,"y")</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="n">
-        <v>45300</v>
+        <v>45291</v>
       </c>
       <c r="B7" s="0" t="n">
         <f aca="false">EDATE(A7,3)</f>
-        <v>45391</v>
+        <v>45382</v>
       </c>
       <c r="C7" s="0" t="n">
+        <f aca="false">EDATE(A7,-2)</f>
+        <v>45230</v>
+      </c>
+      <c r="D7" s="0" t="n">
         <f aca="false">EOMONTH(A7,0)</f>
+        <v>45291</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <f aca="false">EOMONTH(A7,1)</f>
         <v>45322</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="F7" s="0" t="n">
         <f aca="false">DATEDIF(DATE(2020,1,1),A7,"d")</f>
-        <v>1469</v>
+        <v>1460</v>
+      </c>
+      <c r="G7" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A7,"m")</f>
+        <v>47</v>
+      </c>
+      <c r="H7" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A7,"y")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="n">
-        <v>44800</v>
+        <v>43831</v>
       </c>
       <c r="B8" s="0" t="n">
         <f aca="false">EDATE(A8,3)</f>
-        <v>44892</v>
+        <v>43922</v>
       </c>
       <c r="C8" s="0" t="n">
+        <f aca="false">EDATE(A8,-2)</f>
+        <v>43770</v>
+      </c>
+      <c r="D8" s="0" t="n">
         <f aca="false">EOMONTH(A8,0)</f>
-        <v>44804</v>
-      </c>
-      <c r="D8" s="0" t="n">
+        <v>43861</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <f aca="false">EOMONTH(A8,1)</f>
+        <v>43890</v>
+      </c>
+      <c r="F8" s="0" t="n">
         <f aca="false">DATEDIF(DATE(2020,1,1),A8,"d")</f>
-        <v>969</v>
+        <v>0</v>
+      </c>
+      <c r="G8" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A8,"m")</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A8,"y")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="n">
-        <v>45100</v>
+        <v>44561</v>
       </c>
       <c r="B9" s="0" t="n">
         <f aca="false">EDATE(A9,3)</f>
-        <v>45192</v>
+        <v>44651</v>
       </c>
       <c r="C9" s="0" t="n">
+        <f aca="false">EDATE(A9,-2)</f>
+        <v>44500</v>
+      </c>
+      <c r="D9" s="0" t="n">
         <f aca="false">EOMONTH(A9,0)</f>
-        <v>45107</v>
-      </c>
-      <c r="D9" s="0" t="n">
+        <v>44561</v>
+      </c>
+      <c r="E9" s="0" t="n">
+        <f aca="false">EOMONTH(A9,1)</f>
+        <v>44592</v>
+      </c>
+      <c r="F9" s="0" t="n">
         <f aca="false">DATEDIF(DATE(2020,1,1),A9,"d")</f>
-        <v>1269</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
-        <v>45400</v>
-      </c>
-      <c r="B10" s="0" t="n">
-        <f aca="false">EDATE(A10,3)</f>
-        <v>45491</v>
-      </c>
-      <c r="C10" s="0" t="n">
-        <f aca="false">EOMONTH(A10,0)</f>
-        <v>45412</v>
-      </c>
-      <c r="D10" s="0" t="n">
-        <f aca="false">DATEDIF(DATE(2020,1,1),A10,"d")</f>
-        <v>1569</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
-        <v>45500</v>
-      </c>
-      <c r="B11" s="0" t="n">
-        <f aca="false">EDATE(A11,3)</f>
-        <v>45592</v>
-      </c>
-      <c r="C11" s="0" t="n">
-        <f aca="false">EOMONTH(A11,0)</f>
-        <v>45504</v>
-      </c>
-      <c r="D11" s="0" t="n">
-        <f aca="false">DATEDIF(DATE(2020,1,1),A11,"d")</f>
-        <v>1669</v>
+        <v>730</v>
+      </c>
+      <c r="G9" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A9,"m")</f>
+        <v>23</v>
+      </c>
+      <c r="H9" s="0" t="n">
+        <f aca="false">DATEDIF(DATE(2020,1,1),A9,"y")</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>